<commit_message>
Synchronize Phase 1 GitHub roadmap
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R8877b87182114e0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Re3018301444f4385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R133ed017698446a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R86e08a514c0f496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="Rbdab533727074c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R9457d098f04045e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="R2abc036e4e90494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R31bbdff657754787"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="R3928b6064d444bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="Rda582579a0aa414d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R4e9ef6b089854bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R539bc79313914248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R4fa195314ff34d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Ra542773d9d2246cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -727,7 +727,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra79237d3090f4b8d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdcab5b21cd874a6f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -757,7 +757,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R39533c6670384ea5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00eafe76a70a4b86"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2195,7 +2195,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red9dd68a4c1a47d6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R448a1729758a4245"/>
 </x:worksheet>
 </file>
 
@@ -2692,7 +2692,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4598f54d57e4b34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e792898ad7840ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3027,7 +3027,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T6" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/2</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="78" customHeight="1">
@@ -3088,7 +3088,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T7" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/3</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="78" customHeight="1">
@@ -3151,7 +3151,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T8" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/4</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="78" customHeight="1">
@@ -3214,7 +3214,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T9" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/5</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="78" customHeight="1">
@@ -3277,7 +3277,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T10" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/6</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="78" customHeight="1">
@@ -3340,7 +3340,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T11" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/7</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="78" customHeight="1">
@@ -3403,7 +3403,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T12" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/8</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="78" customHeight="1">
@@ -3466,7 +3466,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T13" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/9</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="78" customHeight="1">
@@ -3529,7 +3529,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T14" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="78" customHeight="1">
@@ -3592,7 +3592,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T15" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/11</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="78" customHeight="1">
@@ -3655,7 +3655,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T16" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/12</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="78" customHeight="1">
@@ -3718,7 +3718,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T17" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/13</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="78" customHeight="1">
@@ -3781,7 +3781,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T18" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/14</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="78" customHeight="1">
@@ -3844,7 +3844,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T19" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/15</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="78" customHeight="1">
@@ -3907,7 +3907,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T20" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/16</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="78" customHeight="1">
@@ -3970,7 +3970,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T21" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/17</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="78" customHeight="1">
@@ -4033,7 +4033,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T22" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/18</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="78" customHeight="1">
@@ -4096,7 +4096,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T23" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/19</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="78" customHeight="1">
@@ -4159,7 +4159,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T24" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/20</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="78" customHeight="1">
@@ -4222,7 +4222,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T25" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/21</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="78" customHeight="1">
@@ -4285,7 +4285,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T26" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/22</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="78" customHeight="1">
@@ -4348,7 +4348,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T27" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/23</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="78" customHeight="1">
@@ -4411,7 +4411,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T28" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/24</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="78" customHeight="1">
@@ -4474,7 +4474,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T29" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/25</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="78" customHeight="1">
@@ -4537,7 +4537,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T30" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/26</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="78" customHeight="1">
@@ -4600,7 +4600,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T31" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/27</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="78" customHeight="1">
@@ -4663,7 +4663,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T32" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/28</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="78" customHeight="1">
@@ -4726,7 +4726,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T33" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/29</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="78" customHeight="1">
@@ -4789,7 +4789,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T34" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/30</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="78" customHeight="1">
@@ -4852,7 +4852,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T35" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/31</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="78" customHeight="1">
@@ -4915,7 +4915,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T36" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/32</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="78" customHeight="1">
@@ -4978,7 +4978,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T37" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/33</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="78" customHeight="1">
@@ -5041,7 +5041,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T38" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/34</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="78" customHeight="1">
@@ -5104,7 +5104,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T39" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/35</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="78" customHeight="1">
@@ -5167,7 +5167,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T40" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/36</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="78" customHeight="1">
@@ -5230,7 +5230,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T41" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/37</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="78" customHeight="1">
@@ -5293,7 +5293,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T42" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/38</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="78" customHeight="1">
@@ -5356,7 +5356,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T43" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/39</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="78" customHeight="1">
@@ -5419,7 +5419,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T44" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/40</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="78" customHeight="1">
@@ -5482,7 +5482,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T45" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/41</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="78" customHeight="1">
@@ -5545,7 +5545,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T46" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/42</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="78" customHeight="1">
@@ -5608,7 +5608,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T47" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/43</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="78" customHeight="1">
@@ -5671,7 +5671,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T48" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/44</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="78" customHeight="1">
@@ -5734,7 +5734,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T49" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/45</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="78" customHeight="1">
@@ -5797,7 +5797,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T50" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/46</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="78" customHeight="1">
@@ -5860,7 +5860,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T51" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/47</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="78" customHeight="1">
@@ -5923,7 +5923,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T52" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/48</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="78" customHeight="1">
@@ -5986,7 +5986,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T53" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/49</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="78" customHeight="1">
@@ -6049,7 +6049,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T54" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/50</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="78" customHeight="1">
@@ -6112,7 +6112,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T55" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/51</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="78" customHeight="1">
@@ -6175,7 +6175,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T56" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/52</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="78" customHeight="1">
@@ -6238,7 +6238,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T57" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/53</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="78" customHeight="1">
@@ -6301,7 +6301,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T58" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/54</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="78" customHeight="1">
@@ -6364,7 +6364,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T59" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/55</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="78" customHeight="1">
@@ -6427,7 +6427,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T60" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/56</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="78" customHeight="1">
@@ -6485,7 +6485,7 @@
         <x:v>This planning artifact is complete; it does not claim feature implementation, deployment, production readiness, or release acceptance.</x:v>
       </x:c>
       <x:c r="T61" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/57</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="78" customHeight="1">
@@ -6543,7 +6543,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T62" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/58</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="78" customHeight="1">
@@ -6601,7 +6601,7 @@
         <x:v>Move to Done only when the named task evidence exists; prototype or document intent cannot prove implementation or release completion.</x:v>
       </x:c>
       <x:c r="T63" s="26" t="str">
-        <x:v>Pending GitHub sync</x:v>
+        <x:v>https://github.com/arunpr614/Life-Reflection/issues/59</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6628,7 +6628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R547aa84d63d44953"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff4886df66604b34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15513,7 +15513,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7410a1c695e8406f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14835ba129d2488a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
P0 harden fail-closed execution controls
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R0e6ba4d5bc71492c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Rbb26ca2e8b9c411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R0a589ba9676f4657"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R3dff095b1eed459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R9a22e3f41b1e4747"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R311ea6f78a174215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="R5ec08d1b1d604bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R93554e32559d48b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Rc21812a848ac48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="Re6235de948fc41b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="Rcefcfc4c5ca8491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="Rd8c463c070f54066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R2874b094dbdf4e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Rc1b5140a3de04376"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3c5bc18192e48e7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a81b685a6574b1f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -879,7 +879,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb56a512470e4404f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd49206fc4bb54996"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1298,67 +1298,67 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="D3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="E3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="F3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="G3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="H3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="I3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="J3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="M3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="N3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="O3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="R3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="S3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="T3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="U3" s="16" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-14. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -2362,7 +2362,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c459590b86b413c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d60fc9c52234894"/>
 </x:worksheet>
 </file>
 
@@ -3042,7 +3042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae288e46260422f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb08dfaa3b0254f52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4079,7 +4079,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="F13" s="26" t="str">
-        <x:v>local-synthetic-artifact-authoring-only</x:v>
+        <x:v>future-release-gated</x:v>
       </x:c>
       <x:c r="G13" s="26" t="str">
         <x:v>R0</x:v>
@@ -8669,7 +8669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R189fde69f1ec4a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a57de602ba54d31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17002,7 +17002,7 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="40" customHeight="1">
+    <x:row r="40" ht="73" customHeight="1">
       <x:c r="A40" s="26" t="str">
         <x:v>LID-REF-006</x:v>
       </x:c>
@@ -17065,7 +17065,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="40" customHeight="1">
+    <x:row r="43" ht="47" customHeight="1">
       <x:c r="A43" s="26" t="str">
         <x:v>LID-AIT-002</x:v>
       </x:c>
@@ -17086,7 +17086,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="40" customHeight="1">
+    <x:row r="44" ht="47" customHeight="1">
       <x:c r="A44" s="26" t="str">
         <x:v>LID-AIT-003</x:v>
       </x:c>
@@ -17170,7 +17170,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="40" customHeight="1">
+    <x:row r="48" ht="47" customHeight="1">
       <x:c r="A48" s="26" t="str">
         <x:v>LID-AIT-007</x:v>
       </x:c>
@@ -17233,7 +17233,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="40" customHeight="1">
+    <x:row r="51" ht="47" customHeight="1">
       <x:c r="A51" s="26" t="str">
         <x:v>LID-AIA-003</x:v>
       </x:c>
@@ -17275,7 +17275,7 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="40" customHeight="1">
+    <x:row r="53" ht="47" customHeight="1">
       <x:c r="A53" s="26" t="str">
         <x:v>LID-AIA-005</x:v>
       </x:c>
@@ -17296,7 +17296,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="40" customHeight="1">
+    <x:row r="54" ht="47" customHeight="1">
       <x:c r="A54" s="26" t="str">
         <x:v>LID-AIA-006</x:v>
       </x:c>
@@ -17569,7 +17569,7 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="40" customHeight="1">
+    <x:row r="67" ht="47" customHeight="1">
       <x:c r="A67" s="26" t="str">
         <x:v>LID-OPS-008</x:v>
       </x:c>
@@ -17632,7 +17632,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" ht="40" customHeight="1">
+    <x:row r="70" ht="125" customHeight="1">
       <x:c r="A70" s="26" t="str">
         <x:v>LID-OPS-011</x:v>
       </x:c>
@@ -17695,7 +17695,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" ht="40" customHeight="1">
+    <x:row r="73" ht="60" customHeight="1">
       <x:c r="A73" s="26" t="str">
         <x:v>LID-OPS-014</x:v>
       </x:c>
@@ -17716,7 +17716,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" ht="40" customHeight="1">
+    <x:row r="74" ht="47" customHeight="1">
       <x:c r="A74" s="26" t="str">
         <x:v>LID-OPS-015</x:v>
       </x:c>
@@ -17758,7 +17758,7 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="40" customHeight="1">
+    <x:row r="76" ht="60" customHeight="1">
       <x:c r="A76" s="26" t="str">
         <x:v>LID-OPS-017</x:v>
       </x:c>
@@ -17779,7 +17779,7 @@
         <x:v>17</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="40" customHeight="1">
+    <x:row r="77" ht="125" customHeight="1">
       <x:c r="A77" s="26" t="str">
         <x:v>LID-OPS-018</x:v>
       </x:c>
@@ -17936,7 +17936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aaad7f0db144f03"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf1dd68c8b8345c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18765,21 +18765,6 @@
       <x:c r="C1" s="5" t="str">
         <x:v>Workbook Review Guide and Evidence Boundary</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="E1" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="F1" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="G1" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -18791,21 +18776,6 @@
       <x:c r="C2" s="5" t="str">
         <x:v>Workbook Review Guide and Evidence Boundary</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="str">
-        <x:v>Workbook Review Guide and Evidence Boundary</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
@@ -18814,22 +18784,7 @@
       <x:c r="B3" s="15" t="str">
         <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="str">
-        <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
-      </x:c>
-      <x:c r="D3" s="15" t="str">
-        <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
-      </x:c>
-      <x:c r="E3" s="15" t="str">
-        <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
-      </x:c>
-      <x:c r="F3" s="15" t="str">
-        <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
-      </x:c>
-      <x:c r="G3" s="15" t="str">
-        <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
-      </x:c>
-      <x:c r="H3" s="16" t="str">
+      <x:c r="C3" s="16" t="str">
         <x:v>Use this workbook to review the plan; use the JSON manifest as the edit source. Reconcile any approved change to Markdown, GitHub issues, and the live Project.</x:v>
       </x:c>
     </x:row>
@@ -18857,13 +18812,13 @@
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="41" t="str">
-        <x:v>Canonical source</x:v>
+        <x:v>Source manifest SHA-256</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json</x:v>
+        <x:v>sha256:65060d958a3ac35e312112b180ffc2b7543f63dd02e1d346574c6804f0b64942</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
-        <x:v>Do not use a workbook-only edit as a planning decision.</x:v>
+        <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json — do not use a workbook-only edit as a planning decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
@@ -19066,8 +19021,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H2"/>
-    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A1:C2"/>
+    <x:mergeCell ref="A3:C3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
stage0: harden inert P0 R0 control plane
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R93554e32559d48b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Rc21812a848ac48c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="Re6235de948fc41b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="Rcefcfc4c5ca8491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="Rd8c463c070f54066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R2874b094dbdf4e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Rc1b5140a3de04376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Red13549c38e64843"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="R3d207f13d36a4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R3c40ea8e40cb4506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R384d40defd3e4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R4d6c9fd2524d4f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Rb095448522be415f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Rfe66e19a2c7b46b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a81b685a6574b1f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4ddd00917a34b49"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -879,7 +879,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd49206fc4bb54996"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfc9193a1579e4ee5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1298,67 +1298,67 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="D3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="E3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="F3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="G3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="H3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="I3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="J3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="M3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="N3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="O3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="R3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="S3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="T3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="U3" s="16" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. All 58 task dossiers are currently Incomplete; 0 are execution-authorized. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -2362,7 +2362,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d60fc9c52234894"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R038a2bd8091543ff"/>
 </x:worksheet>
 </file>
 
@@ -3042,7 +3042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb08dfaa3b0254f52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R461d7ca791a64faa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3262,91 +3262,91 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="D3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="E3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="F3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="G3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="H3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="I3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="J3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="M3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="N3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="O3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="R3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="S3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="T3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="U3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="V3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="W3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="X3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="Y3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="Z3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="AA3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="AB3" s="15" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
       <x:c r="AC3" s="16" t="str">
-        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. All current dossiers are Incomplete/Hold; Done on a planning item never implies implementation or deployment.</x:v>
+        <x:v>Every stable task ID projects six P0-prefixed dossier artifacts into its existing issue and Roadmap item. Current control truth: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Done on a planning item never implies implementation or deployment.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -8669,7 +8669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a57de602ba54d31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24fbd751150a4f43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17936,7 +17936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf1dd68c8b8345c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a8e688191984e98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18815,7 +18815,7 @@
         <x:v>Source manifest SHA-256</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>sha256:65060d958a3ac35e312112b180ffc2b7543f63dd02e1d346574c6804f0b64942</x:v>
+        <x:v>sha256:062123c9d79830467a5fbe22a826e4fb769636561a627b8f353d85a7d1a90c69</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
         <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json — do not use a workbook-only edit as a planning decision.</x:v>
@@ -18881,7 +18881,7 @@
         <x:v>Current task readiness</x:v>
       </x:c>
       <x:c r="B13" s="26" t="str">
-        <x:v>58 Incomplete; 0 execution-authorized</x:v>
+        <x:v>58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed</x:v>
       </x:c>
       <x:c r="C13" s="26" t="str">
         <x:v>Artifact generation is not specialist approval; roadmap status is not a start override.</x:v>

</xml_diff>

<commit_message>
fix: close Stage 0 control review vetoes
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Red13549c38e64843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="R3d207f13d36a4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R3c40ea8e40cb4506"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R384d40defd3e4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R4d6c9fd2524d4f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Rb095448522be415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Rfe66e19a2c7b46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4d9d98e3c31d4470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Ra4f52134aa934277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R8d0b4fa8863a485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R04ccdb628fe74d14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R7c6a2740758f4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Ra6e09a397513453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="R12e875af903f4b4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4ddd00917a34b49"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R53c2cef01e044e1e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -879,7 +879,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfc9193a1579e4ee5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33d6b48e9d674127"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1298,67 +1298,67 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="C3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="D3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="E3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="F3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="G3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="H3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="I3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="J3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="L3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="M3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="N3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="O3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="P3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="Q3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="R3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="S3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="T3" s="15" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
       <x:c r="U3" s="16" t="str">
-        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-15. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
+        <x:v>Review workbook generated from PHASE1-ROADMAP-MANIFEST.json on 2026-08-16. Current readiness: 58 Incomplete; 45 Hold + 13 Historical non-authorizing; 0 Ready; 0 execution-allowed. Dates are estimates; evidence gates control delivery.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -2362,7 +2362,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R038a2bd8091543ff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ddc13dca104bfe"/>
 </x:worksheet>
 </file>
 
@@ -3042,7 +3042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R461d7ca791a64faa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb2428d0b2d644cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8669,7 +8669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24fbd751150a4f43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R640c3649cdbd4d2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17936,7 +17936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a8e688191984e98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f572b77d6b46ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18815,7 +18815,7 @@
         <x:v>Source manifest SHA-256</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>sha256:062123c9d79830467a5fbe22a826e4fb769636561a627b8f353d85a7d1a90c69</x:v>
+        <x:v>sha256:27c2a54fbdf9aa45822ad8758741ca64e0c95c554db1457c5ae977d3e7c15b72</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
         <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json — do not use a workbook-only edit as a planning decision.</x:v>

</xml_diff>

<commit_message>
docs: project SPK Gate A proposal
Regenerate the exact three canonical projections for the six-file SPK proposal while preserving Hold, zero execution authority, and the frozen R1-R10 scope.
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4d9d98e3c31d4470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Ra4f52134aa934277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R8d0b4fa8863a485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="R04ccdb628fe74d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R7c6a2740758f4b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Ra6e09a397513453d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="R12e875af903f4b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R701b6e452af64379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="R689102ae6ae04d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R3659043b61544887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="Re1f2e94ce0514a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="Rcb68cd69f49d463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Rce1be630c42544c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Re14137fcbc5643e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R53c2cef01e044e1e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2e763ed1e81f474c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -879,7 +879,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33d6b48e9d674127"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9816b78de844eb1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2362,7 +2362,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ddc13dca104bfe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dd9c4bd7024964"/>
 </x:worksheet>
 </file>
 
@@ -3042,7 +3042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb2428d0b2d644cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c43e2d04a042c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8669,7 +8669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R640c3649cdbd4d2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda3a5ceaaf6e4e3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17936,7 +17936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f572b77d6b46ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29ce15b83ed4ed9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18815,7 +18815,7 @@
         <x:v>Source manifest SHA-256</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>sha256:27c2a54fbdf9aa45822ad8758741ca64e0c95c554db1457c5ae977d3e7c15b72</x:v>
+        <x:v>sha256:8eb460283499fd2f8be3296a6494ff481616f059e684fafc787ef404815a628c</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
         <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json — do not use a workbook-only edit as a planning decision.</x:v>

</xml_diff>

<commit_message>
docs: refresh SPK Gate A proposal projections
## Why
The ratchet-aware SPK Gate A proposal changes six reviewed artifact bytes, so
the canonical register, roadmap manifest, and workbook must bind those exact
bytes while preserving Incomplete, Hold, and executionAllowed=false.
</commit_message>
<xml_diff>
--- a/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
+++ b/outputs/phase1/Life-in-Days-Phase1-Release-Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R701b6e452af64379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="R689102ae6ae04d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R3659043b61544887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="Re1f2e94ce0514a9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="Rcb68cd69f49d463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="Rce1be630c42544c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="Re14137fcbc5643e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R92297ad843274b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="2" r:id="Rf4fa7b0c66ec4a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Tasks" sheetId="3" r:id="R8ecefcc207604c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Timeline" sheetId="4" r:id="Ra3f85d9962134f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirement Map" sheetId="5" r:id="R156ede151ba74d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Gates" sheetId="6" r:id="R7c9d8258b75f43b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Guide" sheetId="7" r:id="R229d7962ea114480"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2e763ed1e81f474c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b78ab0ff05343cd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -879,7 +879,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb9816b78de844eb1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R512579fd21474dc6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2362,7 +2362,7 @@
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Done"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79dd9c4bd7024964"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2c39fd724b84fbb"/>
 </x:worksheet>
 </file>
 
@@ -3042,7 +3042,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96c43e2d04a042c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04f062ee25544859"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8669,7 +8669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda3a5ceaaf6e4e3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97b930fcc9d2407f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17936,7 +17936,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29ce15b83ed4ed9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3090552eaa047d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18815,7 +18815,7 @@
         <x:v>Source manifest SHA-256</x:v>
       </x:c>
       <x:c r="B7" s="26" t="str">
-        <x:v>sha256:8eb460283499fd2f8be3296a6494ff481616f059e684fafc787ef404815a628c</x:v>
+        <x:v>sha256:e312399a16a72a8030e5735413270af989c0295c50b73ce0a9ecf4e02406c166</x:v>
       </x:c>
       <x:c r="C7" s="26" t="str">
         <x:v>docs/project/PHASE1-ROADMAP-MANIFEST.json — do not use a workbook-only edit as a planning decision.</x:v>

</xml_diff>